<commit_message>
Additional analysis including GARCH order robustness and synthetic recovery
</commit_message>
<xml_diff>
--- a/results/consolidated/Consolidated_NF_GARCH_Results.xlsx
+++ b/results/consolidated/Consolidated_NF_GARCH_Results.xlsx
@@ -440,13 +440,13 @@
         <v>11</v>
       </c>
       <c r="F2" t="n">
-        <v>-8536.82881066782</v>
+        <v>-6287.35443106992</v>
       </c>
       <c r="G2" t="n">
-        <v>-8508.24033352615</v>
+        <v>-6259.41251168897</v>
       </c>
       <c r="H2" t="n">
-        <v>4274.41440533391</v>
+        <v>3149.67721553496</v>
       </c>
       <c r="I2" t="n">
         <v>0</v>
@@ -504,13 +504,13 @@
         <v>11</v>
       </c>
       <c r="F4" t="n">
-        <v>-9208.22580628112</v>
+        <v>-6799.03556910042</v>
       </c>
       <c r="G4" t="n">
-        <v>-9179.63732913944</v>
+        <v>-6771.09364971946</v>
       </c>
       <c r="H4" t="n">
-        <v>4610.11290314056</v>
+        <v>3405.51778455021</v>
       </c>
       <c r="I4" t="n">
         <v>0</v>
@@ -536,13 +536,13 @@
         <v>11</v>
       </c>
       <c r="F5" t="n">
-        <v>-8408.52927162422</v>
+        <v>-6175.98575109436</v>
       </c>
       <c r="G5" t="n">
-        <v>-8387.08791376796</v>
+        <v>-6155.02931155864</v>
       </c>
       <c r="H5" t="n">
-        <v>4208.76463581211</v>
+        <v>3092.49287554718</v>
       </c>
       <c r="I5" t="n">
         <v>0</v>

</xml_diff>